<commit_message>
feat: add backend Java classes, configuration files, and Manim animation scripts for Cuckoo Search project
</commit_message>
<xml_diff>
--- a/Results/Compiled Results.xlsx
+++ b/Results/Compiled Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janch\Thesis Project with Antigravity IDE\Binary-Cuckoo-Search-For-Plant-Leaf-Prediction-Fork\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5747FBA4-9DF5-441D-97B8-01270E513DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70C1702-7B92-4C3B-B7EB-D0F9CB41C1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{B2092B7F-C4C0-406D-8CDA-8D1DA8C8D15E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B2092B7F-C4C0-406D-8CDA-8D1DA8C8D15E}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="EDA" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -45,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="64">
   <si>
     <t>ID</t>
   </si>
@@ -135,9 +134,6 @@
   </si>
   <si>
     <t>Dataset_ID</t>
-  </si>
-  <si>
-    <t>Philippines</t>
   </si>
   <si>
     <t>Hybrid Evolution (LÃ©vy Flight + Uniform Crossover Pc=0.8 + Mutation Pm=0.02)</t>
@@ -322,13 +318,13 @@
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -477,21 +473,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -500,13 +497,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>4971</c:v>
+                  <c:v>1907</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1907</c:v>
+                  <c:v>1125</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1125</c:v>
+                  <c:v>4971</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -817,21 +814,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -840,13 +838,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>40</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>33</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15</c:v>
+                  <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1157,21 +1155,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1180,13 +1179,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1497,21 +1496,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1520,13 +1520,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>171</c:v>
+                  <c:v>77</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>171</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1837,21 +1837,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -1860,13 +1861,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>124.28</c:v>
+                  <c:v>57.79</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>57.79</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>124.28</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2177,21 +2178,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -2200,13 +2202,13 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.12529999999999999</c:v>
+                  <c:v>0.1489</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1489</c:v>
+                  <c:v>0.16109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.16109999999999999</c:v>
+                  <c:v>0.12529999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2517,21 +2519,22 @@
             </c:extLst>
           </c:dLbls>
           <c:cat>
-            <c:strRef>
+            <c:numRef>
               <c:f>EDA!$A$2:$A$4</c:f>
-              <c:strCache>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>Philippines</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Flavia</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Swedish</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
-              </c:strCache>
-            </c:strRef>
+              </c:numCache>
+            </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
@@ -2540,13 +2543,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>21</c:v>
+                  <c:v>148</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>148</c:v>
+                  <c:v>66</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>66</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6565,13 +6568,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>800100</xdr:colOff>
+      <xdr:colOff>809625</xdr:colOff>
       <xdr:row>5</xdr:row>
       <xdr:rowOff>4762</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1238250</xdr:colOff>
+      <xdr:colOff>1247775</xdr:colOff>
       <xdr:row>19</xdr:row>
       <xdr:rowOff>80962</xdr:rowOff>
     </xdr:to>
@@ -6637,15 +6640,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>28575</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>800100</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:colOff>771525</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6673,15 +6676,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>790575</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:colOff>866775</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>14287</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1228725</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>166687</xdr:rowOff>
+      <xdr:colOff>1304925</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6709,15 +6712,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1219200</xdr:colOff>
+      <xdr:colOff>1476375</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>80962</xdr:rowOff>
+      <xdr:rowOff>185737</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>257175</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>157162</xdr:rowOff>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>71437</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6785,7 +6788,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6B27232-3A60-4F32-B6D0-78765898BC02}" name="Table1" displayName="Table1" ref="A1:B4" totalsRowShown="0">
   <autoFilter ref="A1:B4" xr:uid="{E6B27232-3A60-4F32-B6D0-78765898BC02}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{8B0426BB-8EE4-43F6-9D42-D1D71C56FE5C}" name="ID" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{8B0426BB-8EE4-43F6-9D42-D1D71C56FE5C}" name="ID" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{F0B5A016-A4BA-4659-B7AA-DF4C3CEA6CE7}" name="Dataset"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6826,7 +6829,7 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{3CC483C9-71F5-4B3E-80D4-CCA99112D3E5}" name="Dataset_ID"/>
     <tableColumn id="2" xr3:uid="{5798481C-D011-4555-91A7-B4BC3A456F7E}" name="Iteration"/>
-    <tableColumn id="3" xr3:uid="{BEDBFE80-04D6-48B0-A65F-8EBB6950ADB3}" name="BestFitnessScore" dataDxfId="2" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{BEDBFE80-04D6-48B0-A65F-8EBB6950ADB3}" name="BestFitnessScore" dataDxfId="5" dataCellStyle="Percent"/>
     <tableColumn id="5" xr3:uid="{F30B1BE3-B213-4984-B614-972E1915A880}" name="SelectedFeatures"/>
     <tableColumn id="6" xr3:uid="{B22BD895-414D-48E3-A0A5-38C58EB91D0F}" name="ReductionRatioPercent" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{A1EFFDB0-07CC-44CA-8B16-C80F69017778}" name="Description"/>
@@ -6841,9 +6844,9 @@
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{D5CE412E-F77F-4400-B8E9-59BA18D987DB}" name="Dataset_ID"/>
     <tableColumn id="2" xr3:uid="{4B411BD3-51CE-496A-A473-8860FD2005D0}" name="Iteration"/>
-    <tableColumn id="3" xr3:uid="{7762C30D-4A20-41AF-9B1A-35D0A651EA79}" name="BestFitnessScore" dataDxfId="1" dataCellStyle="Percent"/>
+    <tableColumn id="3" xr3:uid="{7762C30D-4A20-41AF-9B1A-35D0A651EA79}" name="BestFitnessScore" dataDxfId="2" dataCellStyle="Percent"/>
     <tableColumn id="4" xr3:uid="{EED470DF-32B0-49CD-A526-31FFD7E79FC5}" name="Selected Features"/>
-    <tableColumn id="5" xr3:uid="{4D87F421-D01A-4ED1-B936-FB2899FED5E2}" name="ReductionRatioPercent" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{4D87F421-D01A-4ED1-B936-FB2899FED5E2}" name="ReductionRatioPercent" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{CFC67C6D-B33E-44C7-83FD-EE7E09168CB1}" name="Desciption"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -6854,7 +6857,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{8EDF7B9E-409F-46FC-91A8-F9EDADE340D4}" name="Table6" displayName="Table6" ref="A1:J4" totalsRowShown="0">
   <autoFilter ref="A1:J4" xr:uid="{8EDF7B9E-409F-46FC-91A8-F9EDADE340D4}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J4">
-    <sortCondition descending="1" ref="B1:B4"/>
+    <sortCondition ref="A1:A4"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{6CE34767-A414-4714-A15C-853CAC9F0BCF}" name="Dataset_ID"/>
@@ -7293,28 +7296,28 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
         <v>5</v>
       </c>
       <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
         <v>35</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>36</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>37</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>38</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>39</v>
-      </c>
-      <c r="H1" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -7340,7 +7343,7 @@
         <v>94.401700000000005</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -7366,7 +7369,7 @@
         <v>95.626400000000004</v>
       </c>
       <c r="H3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -7392,7 +7395,7 @@
         <v>96.736400000000003</v>
       </c>
       <c r="H4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -7418,7 +7421,7 @@
         <v>93.404799999999994</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -7444,7 +7447,7 @@
         <v>95.936899999999994</v>
       </c>
       <c r="H6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -7470,7 +7473,7 @@
         <v>96.924000000000007</v>
       </c>
       <c r="H7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -7496,7 +7499,7 @@
         <v>94.819199999999995</v>
       </c>
       <c r="H8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -7522,7 +7525,7 @@
         <v>95.57</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -7548,7 +7551,7 @@
         <v>97.191000000000003</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -7574,7 +7577,7 @@
         <v>94.268600000000006</v>
       </c>
       <c r="H11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -7600,7 +7603,7 @@
         <v>95.859399999999994</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -7626,7 +7629,7 @@
         <v>97.445599999999999</v>
       </c>
       <c r="H13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -7652,7 +7655,7 @@
         <v>93.867900000000006</v>
       </c>
       <c r="H14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
@@ -7678,7 +7681,7 @@
         <v>96.301100000000005</v>
       </c>
       <c r="H15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -7704,7 +7707,7 @@
         <v>97.520799999999994</v>
       </c>
       <c r="H16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -7730,7 +7733,7 @@
         <v>93.965199999999996</v>
       </c>
       <c r="H17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -7756,7 +7759,7 @@
         <v>97.026899999999998</v>
       </c>
       <c r="H18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -7782,7 +7785,7 @@
         <v>97.462500000000006</v>
       </c>
       <c r="H19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -7808,7 +7811,7 @@
         <v>92.925600000000003</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -7834,7 +7837,7 @@
         <v>96.036199999999994</v>
       </c>
       <c r="H21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
@@ -7860,7 +7863,7 @@
         <v>97.551699999999997</v>
       </c>
       <c r="H22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -7886,7 +7889,7 @@
         <v>93.423199999999994</v>
       </c>
       <c r="H23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
@@ -7912,7 +7915,7 @@
         <v>96.6327</v>
       </c>
       <c r="H24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -7938,7 +7941,7 @@
         <v>97.813800000000001</v>
       </c>
       <c r="H25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -9274,13 +9277,13 @@
         <v>21</v>
       </c>
       <c r="D1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E1" t="s">
         <v>23</v>
       </c>
       <c r="F1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -9320,7 +9323,7 @@
         <v>0.312</v>
       </c>
       <c r="F3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -9340,7 +9343,7 @@
         <v>0.312</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -9360,7 +9363,7 @@
         <v>0.33639999999999998</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -9380,7 +9383,7 @@
         <v>0.31009999999999999</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -9400,7 +9403,7 @@
         <v>0.32419999999999999</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -9420,7 +9423,7 @@
         <v>0.32419999999999999</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -9440,7 +9443,7 @@
         <v>0.32419999999999999</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -9460,7 +9463,7 @@
         <v>0.32519999999999999</v>
       </c>
       <c r="F10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -9480,7 +9483,7 @@
         <v>0.32519999999999999</v>
       </c>
       <c r="F11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -9500,7 +9503,7 @@
         <v>0.33350000000000002</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -9520,7 +9523,7 @@
         <v>0.31840000000000002</v>
       </c>
       <c r="F13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -9540,7 +9543,7 @@
         <v>0.31840000000000002</v>
       </c>
       <c r="F14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -9560,7 +9563,7 @@
         <v>0.3276</v>
       </c>
       <c r="F15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -9580,7 +9583,7 @@
         <v>0.3276</v>
       </c>
       <c r="F16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -9600,7 +9603,7 @@
         <v>0.31790000000000002</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -9620,7 +9623,7 @@
         <v>0.33200000000000002</v>
       </c>
       <c r="F18" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -9640,7 +9643,7 @@
         <v>0.33639999999999998</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -9660,7 +9663,7 @@
         <v>0.33639999999999998</v>
       </c>
       <c r="F20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -9680,7 +9683,7 @@
         <v>0.3306</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -9700,7 +9703,7 @@
         <v>0.34129999999999999</v>
       </c>
       <c r="F22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -9740,7 +9743,7 @@
         <v>0.31929999999999997</v>
       </c>
       <c r="F24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -9760,7 +9763,7 @@
         <v>0.31929999999999997</v>
       </c>
       <c r="F25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -9780,7 +9783,7 @@
         <v>0.31929999999999997</v>
       </c>
       <c r="F26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -9800,7 +9803,7 @@
         <v>0.30080000000000001</v>
       </c>
       <c r="F27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -9820,7 +9823,7 @@
         <v>0.30080000000000001</v>
       </c>
       <c r="F28" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -9840,7 +9843,7 @@
         <v>0.30080000000000001</v>
       </c>
       <c r="F29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -9860,7 +9863,7 @@
         <v>0.32469999999999999</v>
       </c>
       <c r="F30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -9880,7 +9883,7 @@
         <v>0.32029999999999997</v>
       </c>
       <c r="F31" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -9900,7 +9903,7 @@
         <v>0.3276</v>
       </c>
       <c r="F32" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -9920,7 +9923,7 @@
         <v>0.33939999999999998</v>
       </c>
       <c r="F33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -9940,7 +9943,7 @@
         <v>0.33939999999999998</v>
       </c>
       <c r="F34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -9960,7 +9963,7 @@
         <v>0.33939999999999998</v>
       </c>
       <c r="F35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -9980,7 +9983,7 @@
         <v>0.32129999999999997</v>
       </c>
       <c r="F36" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -10000,7 +10003,7 @@
         <v>0.33300000000000002</v>
       </c>
       <c r="F37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -10020,7 +10023,7 @@
         <v>0.33300000000000002</v>
       </c>
       <c r="F38" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -10040,7 +10043,7 @@
         <v>0.33739999999999998</v>
       </c>
       <c r="F39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -10060,7 +10063,7 @@
         <v>0.33939999999999998</v>
       </c>
       <c r="F40" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -10080,7 +10083,7 @@
         <v>0.33200000000000002</v>
       </c>
       <c r="F41" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -10100,7 +10103,7 @@
         <v>0.33200000000000002</v>
       </c>
       <c r="F42" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -10120,7 +10123,7 @@
         <v>0.33939999999999998</v>
       </c>
       <c r="F43" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -10160,7 +10163,7 @@
         <v>0.32079999999999997</v>
       </c>
       <c r="F45" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -10180,7 +10183,7 @@
         <v>0.32079999999999997</v>
       </c>
       <c r="F46" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -10200,7 +10203,7 @@
         <v>0.2959</v>
       </c>
       <c r="F47" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -10220,7 +10223,7 @@
         <v>0.2959</v>
       </c>
       <c r="F48" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -10240,7 +10243,7 @@
         <v>0.29149999999999998</v>
       </c>
       <c r="F49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -10260,7 +10263,7 @@
         <v>0.29149999999999998</v>
       </c>
       <c r="F50" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -10280,7 +10283,7 @@
         <v>0.29149999999999998</v>
       </c>
       <c r="F51" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -10300,7 +10303,7 @@
         <v>0.3145</v>
       </c>
       <c r="F52" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -10320,7 +10323,7 @@
         <v>0.3145</v>
       </c>
       <c r="F53" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -10340,7 +10343,7 @@
         <v>0.3145</v>
       </c>
       <c r="F54" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -10360,7 +10363,7 @@
         <v>0.3145</v>
       </c>
       <c r="F55" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -10380,7 +10383,7 @@
         <v>0.3145</v>
       </c>
       <c r="F56" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -10400,7 +10403,7 @@
         <v>0.31840000000000002</v>
       </c>
       <c r="F57" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -10420,7 +10423,7 @@
         <v>0.32179999999999997</v>
       </c>
       <c r="F58" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -10440,7 +10443,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F59" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -10460,7 +10463,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F60" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -10480,7 +10483,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F61" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -10500,7 +10503,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F62" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -10520,7 +10523,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F63" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -10540,7 +10543,7 @@
         <v>0.33150000000000002</v>
       </c>
       <c r="F64" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -10601,99 +10604,99 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>30</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2">
-        <v>4971</v>
+        <v>1907</v>
       </c>
       <c r="C2">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D2">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E2">
-        <v>171</v>
+        <v>77</v>
       </c>
       <c r="F2">
-        <v>124.28</v>
+        <v>57.79</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H2">
         <v>2048</v>
       </c>
       <c r="I2" s="3">
-        <v>0.12529999999999999</v>
+        <v>0.1489</v>
       </c>
       <c r="J2">
-        <v>21</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1907</v>
+        <v>1125</v>
       </c>
       <c r="C3">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="E3">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F3">
-        <v>57.79</v>
+        <v>75</v>
       </c>
       <c r="G3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H3">
         <v>2048</v>
       </c>
       <c r="I3" s="3">
-        <v>0.1489</v>
+        <v>0.16109999999999999</v>
       </c>
       <c r="J3">
-        <v>148</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1125</v>
+        <v>4971</v>
       </c>
       <c r="C4">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="D4">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="E4">
-        <v>75</v>
+        <v>171</v>
       </c>
       <c r="F4">
-        <v>75</v>
+        <v>124.28</v>
       </c>
       <c r="G4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H4">
         <v>2048</v>
       </c>
       <c r="I4" s="3">
-        <v>0.16109999999999999</v>
+        <v>0.12529999999999999</v>
       </c>
       <c r="J4">
-        <v>66</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>